<commit_message>
Source Data workbooks: rebuild Source_Data_ED_Fig3.xlsx from the updated ED Fig 3c table
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/workbooks/Source_Data_ED_Fig3.xlsx
+++ b/source_data/workbooks/Source_Data_ED_Fig3.xlsx
@@ -279,8 +279,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -296,7 +304,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -304,12 +312,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -622,55 +648,55 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -4983,55 +5009,55 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -5123,22 +5149,22 @@
         <v>1</v>
       </c>
       <c r="L3">
-        <v>0.8058</v>
+        <v>0.7894</v>
       </c>
       <c r="M3" t="s">
         <v>68</v>
       </c>
       <c r="N3">
-        <v>0.7981</v>
+        <v>0.782</v>
       </c>
       <c r="O3">
-        <v>0.8138</v>
+        <v>0.7973</v>
       </c>
       <c r="P3">
-        <v>0.7946</v>
+        <v>0.7773</v>
       </c>
       <c r="Q3">
-        <v>0.8171</v>
+        <v>0.8011</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -5229,22 +5255,22 @@
         <v>1</v>
       </c>
       <c r="L5">
-        <v>0.9012</v>
+        <v>0.8637</v>
       </c>
       <c r="M5" t="s">
         <v>68</v>
       </c>
       <c r="N5">
-        <v>0.8913</v>
+        <v>0.852</v>
       </c>
       <c r="O5">
-        <v>0.9103</v>
+        <v>0.875</v>
       </c>
       <c r="P5">
-        <v>0.8855</v>
+        <v>0.8443000000000001</v>
       </c>
       <c r="Q5">
-        <v>0.9143</v>
+        <v>0.8803</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -5759,22 +5785,22 @@
         <v>1</v>
       </c>
       <c r="L15">
-        <v>0.7574</v>
+        <v>0.7499</v>
       </c>
       <c r="M15" t="s">
         <v>68</v>
       </c>
       <c r="N15">
-        <v>0.7369</v>
+        <v>0.7301</v>
       </c>
       <c r="O15">
-        <v>0.7763</v>
+        <v>0.7688</v>
       </c>
       <c r="P15">
-        <v>0.7356</v>
+        <v>0.7288</v>
       </c>
       <c r="Q15">
-        <v>0.7802</v>
+        <v>0.7714</v>
       </c>
     </row>
     <row r="16" spans="1:17">
@@ -5865,22 +5891,22 @@
         <v>1</v>
       </c>
       <c r="L17">
-        <v>0.9224</v>
+        <v>0.9106</v>
       </c>
       <c r="M17" t="s">
         <v>68</v>
       </c>
       <c r="N17">
-        <v>0.9176</v>
+        <v>0.9046</v>
       </c>
       <c r="O17">
-        <v>0.9268</v>
+        <v>0.9161</v>
       </c>
       <c r="P17">
-        <v>0.9142</v>
+        <v>0.9013</v>
       </c>
       <c r="Q17">
-        <v>0.93</v>
+        <v>0.9201</v>
       </c>
     </row>
     <row r="18" spans="1:17">
@@ -5971,22 +5997,22 @@
         <v>1</v>
       </c>
       <c r="L19">
-        <v>0.7689</v>
+        <v>0.7544999999999999</v>
       </c>
       <c r="M19" t="s">
         <v>68</v>
       </c>
       <c r="N19">
-        <v>0.7575</v>
+        <v>0.7433</v>
       </c>
       <c r="O19">
-        <v>0.7785</v>
+        <v>0.7642</v>
       </c>
       <c r="P19">
-        <v>0.7536</v>
+        <v>0.7386</v>
       </c>
       <c r="Q19">
-        <v>0.7835</v>
+        <v>0.7691</v>
       </c>
     </row>
     <row r="20" spans="1:17">
@@ -6077,22 +6103,22 @@
         <v>1</v>
       </c>
       <c r="L21">
-        <v>0.8695000000000001</v>
+        <v>0.8389</v>
       </c>
       <c r="M21" t="s">
         <v>68</v>
       </c>
       <c r="N21">
-        <v>0.8594000000000001</v>
+        <v>0.8278</v>
       </c>
       <c r="O21">
-        <v>0.8801</v>
+        <v>0.8501</v>
       </c>
       <c r="P21">
-        <v>0.8545</v>
+        <v>0.8237</v>
       </c>
       <c r="Q21">
-        <v>0.8846000000000001</v>
+        <v>0.8554</v>
       </c>
     </row>
     <row r="22" spans="1:17">

</xml_diff>